<commit_message>
Modernize dashboard/summary tabs across all 8 products; fix pie chart label corruption
Applies a modern dashboard visual style (solid ribbon title band, unified
light KPI ribbon, flattened chart-feeder tables, filter-panel styling for
selector cells, coordinated bar/line chart palette) to every dashboard and
summary tab across all 8 spreadsheet products, leaving data-entry tabs
untouched.

Also fixes a pre-existing bug where every pie/doughnut chart's data labels
rendered garbled (category + series + value + percent all overlapping)
after the mandatory LibreOffice recalc pass, caused by unset label-type
flags resolving to "show everything" on save. Each chart now explicitly
sets showCatName/showSerName/showVal/showLegendKey to False alongside
showPercent, applied before the workbook's first save so the fix survives
recalculation.
</commit_message>
<xml_diff>
--- a/bill_calendar_template.xlsx
+++ b/bill_calendar_template.xlsx
@@ -222,7 +222,7 @@
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="#,##0.00;;;"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,6 +292,22 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="12"/>
+      <color rgb="FFC9DFC2"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
@@ -301,15 +317,15 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF1F3B21"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF2F5233"/>
+      <sz val="16"/>
+      <color rgb="FF1F3B21"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -336,7 +352,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -346,7 +362,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2F5233"/>
-        <bgColor rgb="FF555555"/>
+        <bgColor rgb="FF1F3B21"/>
       </patternFill>
     </fill>
     <fill>
@@ -357,18 +373,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4C7A47"/>
-        <bgColor rgb="FF555555"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF5EC"/>
-        <bgColor rgb="FFEAF7EC"/>
+        <fgColor rgb="FFDCEAD5"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -388,6 +398,43 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF4C7A47"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF4C7A47"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4C7A47"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF4C7A47"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4C7A47"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color rgb="FF4C7A47"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF4C7A47"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4C7A47"/>
       </bottom>
       <diagonal/>
     </border>
@@ -417,7 +464,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -462,20 +509,48 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -486,11 +561,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -561,8 +636,8 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFEFF5EC"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFC9DFC2"/>
+      <rgbColor rgb="FFDCEAD5"/>
       <rgbColor rgb="FFFFF3CD"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFD09493"/>
@@ -579,11 +654,11 @@
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF4299B0"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF2F5233"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF555555"/>
-      <rgbColor rgb="FF2F5233"/>
+      <rgbColor rgb="FF1F3B21"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -750,12 +825,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
@@ -774,12 +850,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
@@ -798,12 +875,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="3"/>
@@ -822,12 +900,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="4"/>
@@ -846,12 +925,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="5"/>
@@ -870,12 +950,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="6"/>
@@ -894,12 +975,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="7"/>
@@ -918,12 +1000,13 @@
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
-              <c:showLegendKey val="1"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="1"/>
-              <c:showSerName val="1"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>; </c:separator>
+              <c:separator>
+</c:separator>
             </c:dLbl>
             <c:txPr>
               <a:bodyPr wrap="square"/>
@@ -940,12 +1023,13 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="bestFit"/>
-            <c:showLegendKey val="1"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="1"/>
-            <c:separator>; </c:separator>
+            <c:separator>
+</c:separator>
             <c:showLeaderLines val="1"/>
           </c:dLbls>
           <c:cat>
@@ -1070,14 +1154,14 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>176040</xdr:rowOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>165600</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>112320</xdr:rowOff>
+      <xdr:rowOff>98280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1085,7 +1169,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="8226360" y="762120"/>
+        <a:off x="8226360" y="1038240"/>
         <a:ext cx="3959640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3876,90 +3960,95 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="1" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="11" t="n">
+      <c r="B3" s="13" t="n">
         <v>2026</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="11" t="n">
+      <c r="D3" s="15" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="17"/>
+      <c r="F5" s="18" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="n">
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="20" t="n">
         <f aca="false">COUNTIFS('Bill Tracker'!$P$3:$P$52,TRUE(),'Bill Tracker'!$I$3:$I$52,"Yes")</f>
         <v>0</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="20" t="n">
         <f aca="false">COUNTIFS('Bill Tracker'!$P$3:$P$52,TRUE(),'Bill Tracker'!$I$3:$I$52,"No")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="E6" s="17"/>
+      <c r="F6" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="21" t="s">
         <v>53</v>
       </c>
+      <c r="H6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Rent/Mortgage",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -3968,7 +4057,7 @@
       <c r="F8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Utilities",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -3977,7 +4066,7 @@
       <c r="F9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Software &amp; Subscriptions",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -3986,7 +4075,7 @@
       <c r="F10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Insurance",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -3995,7 +4084,7 @@
       <c r="F11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="15" t="n">
+      <c r="G11" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Loan Payment",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -4004,7 +4093,7 @@
       <c r="F12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Marketing",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -4013,7 +4102,7 @@
       <c r="F13" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Supplies",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -4022,7 +4111,7 @@
       <c r="F14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="22" t="n">
         <f aca="false">SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$B$3:$B$52,"Other",'Bill Tracker'!$P$3:$P$52,TRUE())</f>
         <v>0</v>
       </c>
@@ -4039,384 +4128,384 @@
       <c r="G16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="F17" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="23" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="str">
+      <c r="A18" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+0))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+0)))</f>
         <v/>
       </c>
-      <c r="B18" s="17" t="str">
+      <c r="B18" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+1))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+1)))</f>
         <v/>
       </c>
-      <c r="C18" s="17" t="str">
+      <c r="C18" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+2))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+2)))</f>
         <v/>
       </c>
-      <c r="D18" s="17" t="str">
+      <c r="D18" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+3))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+3)))</f>
         <v/>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+4))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+4)))</f>
         <v>1</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+5))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+5)))</f>
         <v>2</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+6))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+6)))</f>
         <v>3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="str">
+      <c r="A19" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+0))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+0)))</f>
         <v/>
       </c>
-      <c r="B19" s="18" t="str">
+      <c r="B19" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+1))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+1)))</f>
         <v/>
       </c>
-      <c r="C19" s="18" t="str">
+      <c r="C19" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+2))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+2)))</f>
         <v/>
       </c>
-      <c r="D19" s="18" t="str">
+      <c r="D19" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+3))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+3)))</f>
         <v/>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E19" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+4))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+4)))</f>
         <v>0</v>
       </c>
-      <c r="F19" s="18" t="n">
+      <c r="F19" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+5))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+5)))</f>
         <v>0</v>
       </c>
-      <c r="G19" s="18" t="n">
+      <c r="G19" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+6))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+6)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+7))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+7)))</f>
         <v>4</v>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+8))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+8)))</f>
         <v>5</v>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+9))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+9)))</f>
         <v>6</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+10))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+10)))</f>
         <v>7</v>
       </c>
-      <c r="E20" s="17" t="n">
+      <c r="E20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+11))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+11)))</f>
         <v>8</v>
       </c>
-      <c r="F20" s="17" t="n">
+      <c r="F20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+12))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+12)))</f>
         <v>9</v>
       </c>
-      <c r="G20" s="17" t="n">
+      <c r="G20" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+13))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+13)))</f>
         <v>10</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="n">
+      <c r="A21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+7))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+7)))</f>
         <v>0</v>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+8))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+8)))</f>
         <v>0</v>
       </c>
-      <c r="C21" s="18" t="n">
+      <c r="C21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+9))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+9)))</f>
         <v>0</v>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+10))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+10)))</f>
         <v>0</v>
       </c>
-      <c r="E21" s="18" t="n">
+      <c r="E21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+11))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+11)))</f>
         <v>0</v>
       </c>
-      <c r="F21" s="18" t="n">
+      <c r="F21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+12))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+12)))</f>
         <v>0</v>
       </c>
-      <c r="G21" s="18" t="n">
+      <c r="G21" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+13))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+13)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="n">
+      <c r="A22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+14))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+14)))</f>
         <v>11</v>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+15))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+15)))</f>
         <v>12</v>
       </c>
-      <c r="C22" s="17" t="n">
+      <c r="C22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+16))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+16)))</f>
         <v>13</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+17))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+17)))</f>
         <v>14</v>
       </c>
-      <c r="E22" s="17" t="n">
+      <c r="E22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+18))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+18)))</f>
         <v>15</v>
       </c>
-      <c r="F22" s="17" t="n">
+      <c r="F22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+19))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+19)))</f>
         <v>16</v>
       </c>
-      <c r="G22" s="17" t="n">
+      <c r="G22" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+20))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+20)))</f>
         <v>17</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="n">
+      <c r="A23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+14))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+14)))</f>
         <v>0</v>
       </c>
-      <c r="B23" s="18" t="n">
+      <c r="B23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+15))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+15)))</f>
         <v>0</v>
       </c>
-      <c r="C23" s="18" t="n">
+      <c r="C23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+16))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+16)))</f>
         <v>0</v>
       </c>
-      <c r="D23" s="18" t="n">
+      <c r="D23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+17))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+17)))</f>
         <v>0</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+18))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+18)))</f>
         <v>0</v>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="F23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+19))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+19)))</f>
         <v>0</v>
       </c>
-      <c r="G23" s="18" t="n">
+      <c r="G23" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+20))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+20)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+21))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+21)))</f>
         <v>18</v>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+22))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+22)))</f>
         <v>19</v>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+23))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+23)))</f>
         <v>20</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+24))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+24)))</f>
         <v>21</v>
       </c>
-      <c r="E24" s="17" t="n">
+      <c r="E24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+25))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+25)))</f>
         <v>22</v>
       </c>
-      <c r="F24" s="17" t="n">
+      <c r="F24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+26))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+26)))</f>
         <v>23</v>
       </c>
-      <c r="G24" s="17" t="n">
+      <c r="G24" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+27))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+27)))</f>
         <v>24</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="n">
+      <c r="A25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+21))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+21)))</f>
         <v>0</v>
       </c>
-      <c r="B25" s="18" t="n">
+      <c r="B25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+22))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+22)))</f>
         <v>0</v>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+23))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+23)))</f>
         <v>0</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+24))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+24)))</f>
         <v>0</v>
       </c>
-      <c r="E25" s="18" t="n">
+      <c r="E25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+25))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+25)))</f>
         <v>0</v>
       </c>
-      <c r="F25" s="18" t="n">
+      <c r="F25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+26))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+26)))</f>
         <v>0</v>
       </c>
-      <c r="G25" s="18" t="n">
+      <c r="G25" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+27))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+27)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="n">
+      <c r="A26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+28))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+28)))</f>
         <v>25</v>
       </c>
-      <c r="B26" s="17" t="n">
+      <c r="B26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+29))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+29)))</f>
         <v>26</v>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+30))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+30)))</f>
         <v>27</v>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+31))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+31)))</f>
         <v>28</v>
       </c>
-      <c r="E26" s="17" t="n">
+      <c r="E26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+32))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+32)))</f>
         <v>29</v>
       </c>
-      <c r="F26" s="17" t="n">
+      <c r="F26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+33))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+33)))</f>
         <v>30</v>
       </c>
-      <c r="G26" s="17" t="n">
+      <c r="G26" s="24" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+34))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+34)))</f>
         <v>31</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="n">
+      <c r="A27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+28))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+28)))</f>
         <v>0</v>
       </c>
-      <c r="B27" s="18" t="n">
+      <c r="B27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+29))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+29)))</f>
         <v>0</v>
       </c>
-      <c r="C27" s="18" t="n">
+      <c r="C27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+30))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+30)))</f>
         <v>0</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+31))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+31)))</f>
         <v>0</v>
       </c>
-      <c r="E27" s="18" t="n">
+      <c r="E27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+32))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+32)))</f>
         <v>0</v>
       </c>
-      <c r="F27" s="18" t="n">
+      <c r="F27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+33))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+33)))</f>
         <v>0</v>
       </c>
-      <c r="G27" s="18" t="n">
+      <c r="G27" s="25" t="n">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+34))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+34)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="str">
+      <c r="A28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+35))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+35)))</f>
         <v/>
       </c>
-      <c r="B28" s="17" t="str">
+      <c r="B28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+36))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+36)))</f>
         <v/>
       </c>
-      <c r="C28" s="17" t="str">
+      <c r="C28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+37))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+37)))</f>
         <v/>
       </c>
-      <c r="D28" s="17" t="str">
+      <c r="D28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+38))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+38)))</f>
         <v/>
       </c>
-      <c r="E28" s="17" t="str">
+      <c r="E28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+39))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+39)))</f>
         <v/>
       </c>
-      <c r="F28" s="17" t="str">
+      <c r="F28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+40))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+40)))</f>
         <v/>
       </c>
-      <c r="G28" s="17" t="str">
+      <c r="G28" s="24" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+41))&lt;&gt;$D$3,"",DAY((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+41)))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="str">
+      <c r="A29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+35))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+35)))</f>
         <v/>
       </c>
-      <c r="B29" s="18" t="str">
+      <c r="B29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+36))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+36)))</f>
         <v/>
       </c>
-      <c r="C29" s="18" t="str">
+      <c r="C29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+37))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+37)))</f>
         <v/>
       </c>
-      <c r="D29" s="18" t="str">
+      <c r="D29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+38))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+38)))</f>
         <v/>
       </c>
-      <c r="E29" s="18" t="str">
+      <c r="E29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+39))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+39)))</f>
         <v/>
       </c>
-      <c r="F29" s="18" t="str">
+      <c r="F29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+40))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+40)))</f>
         <v/>
       </c>
-      <c r="G29" s="18" t="str">
+      <c r="G29" s="25" t="str">
         <f aca="false">IF(MONTH((DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+41))&lt;&gt;$D$3,"",SUMIFS('Bill Tracker'!$C$3:$C$52,'Bill Tracker'!$R$3:$R$52,(DATE($B$3,$D$3,1)-(WEEKDAY(DATE($B$3,$D$3,1))-1)+41)))</f>
         <v/>
       </c>

</xml_diff>